<commit_message>
Add Next.js web app for social media automation
Full-stack web interface replacing the Python CLI:
- Form-based UI with rich text editor for creating/editing posts
- Multi-platform posting (Mastodon, LinkedIn, Facebook, Instagram)
- Video and image support across all platforms
- Cron endpoint for scheduled post publishing (/api/cron)
- Token management with extend/permanent token support
- Simple password-gated auth with cookie sessions
- Settings page for connecting/disconnecting social accounts
- Auto-refreshing dashboard (15s polling)
- Vercel deployment ready with cron config

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/posts_template.xlsx
+++ b/posts_template.xlsx
@@ -2,22 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18020" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Posts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,8 +25,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -39,7 +49,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
+        <fgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -52,17 +62,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -425,8 +438,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
@@ -492,155 +505,190 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Hello world</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>instagram</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>mastodon</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Image Test Post 3</t>
+          <t>Facebook Test</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Testing image attachment with a freely accessible image.</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>https://picsum.photos/400/300</t>
+          <t>Hello from the lab automation system! Testing Facebook posting.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>mastodon</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>facebook</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Facebook Test</t>
+          <t>Facebook Image Test</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hello from the lab automation system! Testing Facebook posting.</t>
+          <t>Check out this photo from our lab! Testing image posting via automation.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/800/600</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>facebook</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Facebook Image Test</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Check out this photo from our lab! Testing image posting via automation.</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>https://picsum.photos/800/600</t>
+          <t>LinkedIn Test</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>The 7th Conference on AI Music Creativity will take place 16–18 September 2026. Companies like @Apple and @Google are pushing the boundaries of AI in creative fields. Excited to see what innovations emerge!
+#AI #Music #Apple #Innovation</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>facebook</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>linkedin</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LinkedIn Test</t>
+          <t>Lab Research Update</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Excited to share updates from our lab! Testing automated LinkedIn posting.</t>
+          <t>Exciting research happening at our lab! Inspired by @Apple Vision Pro and spatial computing, we are exploring new ways AI can enhance creative workflows.
+#AI #Research #Apple #Innovation #Lab</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://picsum.photos/800/600</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>linkedin</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Lab Research Update</t>
+          <t>AI in Healthcare</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Exciting research happening at our lab! We are pushing the boundaries of what is possible with AI and creative technology. Stay tuned for more updates.
-#AI #Research #Innovation #Lab</t>
+          <t>From @Apple Health to diagnostic AI, artificial intelligence is transforming healthcare delivery. The future of personalized medicine is here.
+What area excites you most?
+#AI #Healthcare #Apple #Innovation</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -650,7 +698,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -658,13 +706,62 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>YES</t>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Team Collaboration Tips</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Great teams don't just happen — they are built. Here are 3 things we practice daily:
+1. Transparent communication
+2. Async-first workflows
+3. Celebrate small wins
+What works for your team?
+#Leadership #Teamwork #Culture</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Open Source Contribution</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>We just open-sourced our social media automation toolkit! Manage posts across Instagram, Facebook, Mastodon, and LinkedIn from a single spreadsheet.
+Check it out and let us know what you think.
+#OpenSource #Automation #SocialMedia #Python</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>linkedin</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" tooltip="https://aimc2026.org/home" display="https://aimc2026.org/home" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>